<commit_message>
Add vendor file edit modal, ignore Excel lock files
- Replace the bare Delete button in Admin's Vendor Files table with an
  Edit action that opens a modal for replacing or deleting the file.
- Ignore transient Excel lock files (~$*.xlsx) so they never get committed.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Thread Chart/4imprint Thread Charts.xlsx
+++ b/Thread Chart/4imprint Thread Charts.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://idynamicsindia-my.sharepoint.com/personal/mahesh_mohan_idynamics_com/Documents/Thread chart new/Thread chart Nov 23/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\PMS_RA Color Finder\Thread Chart\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="3" documentId="13_ncr:1_{913BB756-1A6A-4F2D-90E7-D4018D306BC6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{9F38C8CB-46CA-4AEB-9C65-B5FA9390BE5F}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{82EA7B92-D68F-463F-A7F9-2D52911764D0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="37275" yWindow="1830" windowWidth="17820" windowHeight="12735" tabRatio="548" xr2:uid="{EC9DC14C-69D5-4A56-AA26-CD1097EEDA67}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="548" activeTab="1" xr2:uid="{EC9DC14C-69D5-4A56-AA26-CD1097EEDA67}"/>
   </bookViews>
   <sheets>
     <sheet name="Robison Anton SS Rayon" sheetId="2" r:id="rId1"/>
@@ -7664,10 +7664,6 @@
 </xdr:wsDr>
 </file>
 
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
-</file>
-
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
 <a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
   <a:themeElements>
@@ -16700,11 +16696,11 @@
         <v>360</v>
       </c>
       <c r="D6" s="610">
-        <v>9103</v>
+        <v>9999</v>
       </c>
       <c r="E6" s="355"/>
       <c r="F6" s="3">
-        <v>324</v>
+        <v>3221</v>
       </c>
       <c r="G6" s="3">
         <v>156</v>
@@ -17537,11 +17533,11 @@
         <v>360</v>
       </c>
       <c r="D37" s="610">
-        <v>5603</v>
+        <v>5555</v>
       </c>
       <c r="E37" s="18"/>
       <c r="F37" s="3">
-        <v>281</v>
+        <v>2222</v>
       </c>
       <c r="G37" s="3">
         <v>0</v>

</xml_diff>